<commit_message>
Gitignore the SQLite CRM file, track the Excel export instead
data/outreach.sqlite3 has never been part of this repo's history —
checking git log, only data/crm_database.xlsx has ever been committed
(via the existing GitHub Action's "Update CRM Database" commits, which
only ever adds the .xlsx). Following that established convention
rather than starting to track the binary SQLite file: gitignored it,
and committed a fresh Excel export reflecting current CRM state (6
Indonesia prospects claimed for sending, not yet sent).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:R7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -482,6 +482,395 @@
           <t>date_contacted</t>
         </is>
       </c>
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>meeting_status</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>meeting_time</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
+        <is>
+          <t>proposed_slots_json</t>
+        </is>
+      </c>
+      <c r="Q1" t="inlineStr">
+        <is>
+          <t>meeting_notes</t>
+        </is>
+      </c>
+      <c r="R1" t="inlineStr">
+        <is>
+          <t>meeting_updated</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>contact@zankore.com</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr"/>
+      <c r="C2" t="inlineStr"/>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>ZanKore (Indosat, Ooredoo Group, Nokia, Nvidia)</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>web_research: https://zankore.com/ — Indosat, Ooredoo Group, Nokia and Nvidia launched Zankore, targeting 1GW of Nvidia DSX AI Factory capacity in Indonesia, with an initial ~200MW live in Jakarta by H1 2027</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>sending</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
+        <v>1</v>
+      </c>
+      <c r="J2" t="inlineStr"/>
+      <c r="K2" t="inlineStr"/>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>2026-09-05T20:38:49+00:00</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr"/>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr"/>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr"/>
+      <c r="R2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>corpsec@dci-indonesia.com</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Corporate Secretary / Investor Relations</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>DCI Indonesia</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>web_research: https://dci-indonesia.com/news/dci-indonesia-inaugurates-e2-surabaya-expanding-its-platform-to-eastern-indonesia — Inaugurated E2 Surabaya (9MW IT load), its first data center in Eastern Indonesia, and separately raised a $980M loan to fund AI-era capacity expansion</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>sending</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
+        <v>1</v>
+      </c>
+      <c r="J3" t="inlineStr"/>
+      <c r="K3" t="inlineStr"/>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>2026-09-05T20:38:49+00:00</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr"/>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr"/>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr"/>
+      <c r="R3" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>dina.yang@digitaledgedc.com</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Dina Yang</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Associate Director, Corporate Communications</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Digital Edge Indonesia</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>web_research: https://www.digitaledgedc.com/resources/newsroom/digital-edge-4-5b-cgk-500mw-ai-ready-hyperscale-campus-indonesia/ — Announced a $4.5B investment in CGK Campus, a 500MW (scaling to 1GW) AI-ready hyperscale data center in Bekasi featuring direct-to-chip liquid cooling and a 1.25 target PUE</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>sending</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
+        <v>1</v>
+      </c>
+      <c r="J4" t="inlineStr"/>
+      <c r="K4" t="inlineStr"/>
+      <c r="L4" t="inlineStr">
+        <is>
+          <t>2026-09-05T20:38:49+00:00</t>
+        </is>
+      </c>
+      <c r="M4" t="inlineStr"/>
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr"/>
+      <c r="P4" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q4" t="inlineStr"/>
+      <c r="R4" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>sales.admin@neutradc.com</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr"/>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>NeutraDC (Telkom Indonesia)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>web_research: https://www.neutradc.com/news/60643/data-center-fully-secured-before-launch-telkom-indonesia-accelerates-expansion-of-neutradc-capacity-in-batam — Accelerating NeutraDC AI data center capacity in Batam (Nxera, 18MW initial phase scaling to 54MW) plus a 200MW Cikarang hyperscale expansion secured via a PLN power deal</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>sending</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
+        <v>1</v>
+      </c>
+      <c r="J5" t="inlineStr"/>
+      <c r="K5" t="inlineStr"/>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>2026-09-05T20:38:49+00:00</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr"/>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr"/>
+      <c r="P5" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q5" t="inlineStr"/>
+      <c r="R5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>support@bdxworld.com</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
+      <c r="C6" t="inlineStr"/>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>BDx Indonesia (Big Data Exchange)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>web_research: https://www.bdxworld.com/locations/indonesia/ — Building BDx Jakarta CGK3, one of Indonesia's first liquid-cooled AI data center campuses, plus a $320M loan-backed expansion of CGK4/CGK5 to 1.2GVA for high-density AI workloads</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>sending</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
+        <v>1</v>
+      </c>
+      <c r="J6" t="inlineStr"/>
+      <c r="K6" t="inlineStr"/>
+      <c r="L6" t="inlineStr">
+        <is>
+          <t>2026-09-05T20:38:49+00:00</t>
+        </is>
+      </c>
+      <c r="M6" t="inlineStr"/>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr"/>
+      <c r="P6" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q6" t="inlineStr"/>
+      <c r="R6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>support@firmus.co</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr"/>
+      <c r="C7" t="inlineStr"/>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Firmus Technologies</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>web_research: https://firmus.co/newsroom/firmus-to-build-170-000-gpu-ai-factor-y-campus-with-nvidia-for-global-ai-natives — Partnering with Nvidia on an 8-year deal to build a 360MW, 170,000-GPU AI Factory campus in Batam, Indonesia, going live Q1 2027</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>sending</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
+        <v>1</v>
+      </c>
+      <c r="J7" t="inlineStr"/>
+      <c r="K7" t="inlineStr"/>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>2026-09-05T20:38:49+00:00</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr"/>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr"/>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr"/>
+      <c r="R7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Batch 4: research + send 10 more Indonesia prospects, audit one domain flag
Added 10 audited prospects from batch 4 research (Datacomm Diangraha,
Biznet Gio Nusantara, Equinix Indonesia, AREA31, SpaceDC, UGM, NEX
Datacenter, AWS Indonesia, Zettagrid, Wowrack) and sent all 10 live via
Gmail. CRM now at 22 sent total. Contact-form fills for the same 10
companies plus 2 form-only entries (AGIT, Oracle Indonesia) running as a
separate step.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R13"/>
+  <dimension ref="A1:R23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1340,6 +1340,714 @@
       <c r="Q13" t="inlineStr"/>
       <c r="R13" t="inlineStr"/>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>aws-pr@amazon.com</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Press/Media Relations</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>Amazon Web Services (AWS) Indonesia</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>web_research: https://www.amazon.jobs/en/jobs/3187721/dceo-facility-manager-indonesia-data-center-engineering-operations — Actively hiring a DCEO Facility Manager for its Indonesia data center cluster to manage electrical/mechanical critical infrastructure (chillers, cooling towers, CRAH units, generators, UPS) supporting the AWS Asia Pacific (Jakarta) Region</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>1a0812521f679104</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr"/>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:11:32+00:00</t>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr"/>
+      <c r="P14" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q14" t="inlineStr"/>
+      <c r="R14" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>humas@ugm.ac.id</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr"/>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>Public Relations (Humas)</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Universitas Gadjah Mada</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>web_research: https://ugm.ac.id/en/news/ugm-partners-with-nvidia-and-indosat-to-advance-ai-research/ — Hosting the UGM Indosat NVIDIA AI Technology Center (opened August 2026), Indonesia's first university AI center, with an NVIDIA DGX Station AI supercomputer placed at the Faculty of Engineering and Faculty of Mathematics and Natural Sciences</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
+        <v>1</v>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>1a08124e1a4af6af</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr"/>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:11:15+00:00</t>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr"/>
+      <c r="P15" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q15" t="inlineStr"/>
+      <c r="R15" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>info@datacomm.co.id</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Tan Wie Tjin</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>President Director &amp; Founder</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Datacomm Diangraha</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>web_research: https://www.prnewswire.com/news-releases/nokia-blaize-and-datacomm-diangraha-unite-to-deliver-hybrid-ai-inference-across-indonesia-and-southeast-asia-302755505.html — Announced (April 2026) a strategic alliance with Nokia and Blaize to deploy hybrid AI inference infrastructure across Indonesia, with Datacomm's own leadership stating data centers must evolve toward GPU infrastructure to meet enterprise/public-sector AI demand</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
+        <v>1</v>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>1a0812444a22266b</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr"/>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:36+00:00</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr"/>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr"/>
+      <c r="R16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>info@nexdatacenter.com</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr"/>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Info/Sales</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NEX Datacenter (PT CBN Nusantara)</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>web_research: https://www.nexdatacenter.com/locations/ — Operates multiple Tier III colocation facilities in Jakarta CBD (Cyber 2 Tower, Menara Tendean) purpose-built for high-density deployments up to 10kVA per rack, part of Indonesia's growing carrier-neutral colocation cluster</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
+        <v>1</v>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>1a081250146ef7f5</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr"/>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:11:24+00:00</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr"/>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr"/>
+      <c r="R17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>info@spacedc.com</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr"/>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>General Enquiries</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SpaceDC</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>web_research: https://spacedc.com/spacedcs-data-center-campus-first-in-indonesia-to-feature-advanced-cooling-technology-to-facilitate-energy-and-space-efficiencies/ — JAK1 Jakarta campus is first in Indonesia to feature advanced cooling technology (Vertiv thermal walls, N+1 high-efficiency air-cooled chillers with cogeneration absorption chillers, hot-aisle containment) with water-cooled racks up to 50kW each</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
+        <v>1</v>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>1a08124bed10cf44</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr"/>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:11:07+00:00</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr"/>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr"/>
+      <c r="R18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>press@equinix.com</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Haris Izmee</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Managing Director, Indonesia</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>Equinix Indonesia</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>web_research: https://newsroom.equinix.com/2025-05-15-Equinix-Unveils-Its-First-AI-Ready-Data-Center-with-Dense-Ecosystem-in-Jakarta — Inaugurated JK1, its first AI-ready IBX data center in Jakarta (JV with PT Astra International), with phase two adding liquid cooling and Cooling Array technology to support higher-density AI workloads at a target PUE of 1.41</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
+        <v>1</v>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>1a0812481201f6c1</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr"/>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:51+00:00</t>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr"/>
+      <c r="P19" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q19" t="inlineStr"/>
+      <c r="R19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>sales@area31.id</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr"/>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>AREA31 Datacenter &amp; Teleport Facilities</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/area31-to-invest-675m-in-depok-indonesia-data-center/ — Committing ~$67.5M over five years to expand its Depok (Cimanggis) hyperscale campus, including a new Data Hall 2 (150+ racks, 600kW capacity) at its AI-ready, carrier-neutral RATED 3 facility</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
+        <v>1</v>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>1a08124a14825778</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr"/>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:59+00:00</t>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr"/>
+      <c r="P20" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q20" t="inlineStr"/>
+      <c r="R20" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>sales@biznetgio.com</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr"/>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Biznet Gio Nusantara</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>web_research: https://www.biznetgio.com/en/product/neo-gpu — Launched NEO GPU cloud service offering up to 8x NVIDIA H200 GPUs per instance (3,958 TFLOPS, 1,128GB HBM3e with NVLink) for AI training/inference workloads hosted in its Indonesia data centers</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
+        <v>1</v>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>1a08124631a7bea9</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr"/>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:43+00:00</t>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr"/>
+      <c r="P21" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q21" t="inlineStr"/>
+      <c r="R21" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>sales@wowrack.co.id</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr"/>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>Wowrack Indonesia</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>web_research: https://www.wowrack.com/en-us/blog/colocation/gpu-as-a-service/ — Offers GPU-as-a-Service (GPUaaS) out of its Jakarta and Surabaya data centers, giving AI teams on-demand access to GPU capacity without their own hardware investment, amid rising Indonesian AI/GPU infrastructure demand</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
+        <v>1</v>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>1a0812564d07ef3e</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr"/>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:11:50+00:00</t>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr"/>
+      <c r="P22" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q22" t="inlineStr"/>
+      <c r="R22" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>sales@zettagrid.id</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr"/>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>Sales</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>Zettagrid Indonesia</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>web_research: https://www.zettagrid.id/gpu-vworkstations/ — Offers Enterprise AI Instances powered by Dell servers with NVIDIA A100 and H100 GPUs, plus GPU vWorkstations, run on VMware infrastructure with NVIDIA AI Enterprise in its Indonesia data center</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
+        <v>1</v>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>1a0812541647810f</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr"/>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:10:26+00:00</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>2026-09-08T13:11:40+00:00</t>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr"/>
+      <c r="P23" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q23" t="inlineStr"/>
+      <c r="R23" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Batch 5: research + send 4 more Indonesia prospects, 11 form-only queued
WebFetch was blocked again this session, so Scout worked WebSearch-only
and applied the domain-match rule strictly — only 4 of ~25 companies
evaluated had a real, verifiable, domain-matched email (Indosat Ooredoo
Hutchison, Peruri, Telin, GDS Indonesia), all sent live via Gmail. The
other 7 real leads found (PLN Icon Plus, Telkomsigma, Sentral Data
Nusantara, BNI, Aslan Energy Capital, SEAX Global, BINUS AI R&D Center)
only had guessable/unverifiable emails, so they're queued contact-form-only
rather than guessed at. CRM now at 26 sent total. Contact-form fills for
today's 11 queued companies running as a separate step.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R23"/>
+  <dimension ref="A1:R27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2048,6 +2048,270 @@
       <c r="Q23" t="inlineStr"/>
       <c r="R23" t="inlineStr"/>
     </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>contact@peruri.co.id</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr"/>
+      <c r="C24" t="inlineStr"/>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Peruri</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>web_research: https://www.lintasarta.net/en/news/lintasarta-presents-gpu-merdeka-an-advanced-sovereign-ai-cloud-for-indonesia-powered-by-nvidia-ai/ — Peruri's Digital Business Director Farah Fitria Rahmayanti participated in the launch of GPU Merdeka, Indonesia's NVIDIA-powered sovereign AI GPU-as-a-Service cloud, indicating Peruri is adopting GPU-accelerated AI infrastructure for its state digital security services</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
+        <v>1</v>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>1a0850fb72832e3a</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr"/>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t>2026-09-09T07:26:21+00:00</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>2026-09-09T07:26:38+00:00</t>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr"/>
+      <c r="P24" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q24" t="inlineStr"/>
+      <c r="R24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>corcomm@telin.net</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
+      <c r="C25" t="inlineStr"/>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Telin</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/telin-and-bw-digital-partner-on-batam-singapore-subsea-cable/ — Telin is building the new Nongsa-Changi Cable and INSICA subsea cable systems (landed Jul 2026 / ready Q4 2026) specifically to carry the surge in data-center-to-data-center traffic between Batam and Singapore, signaling major new DC interconnection capacity build-out</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
+        <v>1</v>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>1a0850fd78650da2</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr"/>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>2026-09-09T07:26:21+00:00</t>
+        </is>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>2026-09-09T07:26:45+00:00</t>
+        </is>
+      </c>
+      <c r="N25" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O25" t="inlineStr"/>
+      <c r="P25" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q25" t="inlineStr"/>
+      <c r="R25" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>corporate.communications@ioh.co.id</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr"/>
+      <c r="C26" t="inlineStr"/>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Indosat Ooredoo Hutchison</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>web_research: https://blogs.nvidia.com/blog/indonesia-ai-center-of-excellence — Building Indonesia's AI Center of Excellence with NVIDIA (Blackwell GPUs, NVIDIA Cloud Partner reference architectures) and Cisco (announced July 2025); also invested ~$200M in a Surakarta AI data center with NVIDIA and formed the Raia Grid JV to assemble NVIDIA GPUs domestically in Indonesia starting Dec 2026</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
+        <v>1</v>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>1a0850f96f15772b</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr"/>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>2026-09-09T07:26:21+00:00</t>
+        </is>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>2026-09-09T07:26:30+00:00</t>
+        </is>
+      </c>
+      <c r="N26" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O26" t="inlineStr"/>
+      <c r="P26" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q26" t="inlineStr"/>
+      <c r="R26" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>marketing@gds-services.com</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
+      <c r="C27" t="inlineStr"/>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>GDS Indonesia</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/gds-partners-with-indonesias-sovereign-wealth-fund-for-batam-data-center-campus/ — GDS Holdings and Indonesia's sovereign wealth fund (INA) formed a JV building a 28MW hyperscale data center campus at Nongsa Digital Park, Batam, integrating GDS's Smart DC solution</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
+        <v>1</v>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>1a0850ff74446503</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr"/>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>2026-09-09T07:26:21+00:00</t>
+        </is>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>2026-09-09T07:26:54+00:00</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O27" t="inlineStr"/>
+      <c r="P27" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q27" t="inlineStr"/>
+      <c r="R27" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Batch 6: research + send 2 more Indonesia prospects, fix double-period bug
WebFetch was blocked again, so Scout worked WebSearch-only and dropped 2
candidate emails that failed a second cross-check rather than guessing.
Only 2 of ~27 companies evaluated had a real, verifiable, domain-matched
email (Intiland/DC Land, Matrix NAP Info), both sent live via Gmail. 10
more real leads (BCA, Nongsa Digital Park, TrendAI, Allo Bank, RAIA Grid,
ByteDance, Microsoft Indonesia, Google Cloud Indonesia, BSI, Dukcapil)
only had generic/unverifiable contact emails, so they're queued
contact-form-only. CRM now at 28 sent total.

Also fixed a copy bug in generate_personalized_email: when a Source
signal already ended in a period, the opener line got a double period
("...demand.."). Stripped the trailing period before appending one.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R27"/>
+  <dimension ref="A1:R29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2312,6 +2312,146 @@
       <c r="Q27" t="inlineStr"/>
       <c r="R27" t="inlineStr"/>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>investor@intiland.com</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr"/>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Investor Relations</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Intiland (DC Land)</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>web_research: https://ekonomi.bisnis.com/read/20260206/47/1950875/intiland-dild-luncurkan-data-center-land-di-surabaya-berkapasitas-3mw — Intiland (via JV PT Inti Arunika Persada with ION Network) launched DC Land data center at Intiland Tower Surabaya Feb 2026, live at 3MW with ~50% capacity already occupied, targeting expansion to 30MW to serve East Indonesia demand.</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
+        <v>1</v>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>1a08a33a21b90f3b</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr"/>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:23:50+00:00</t>
+        </is>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:23:58+00:00</t>
+        </is>
+      </c>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O28" t="inlineStr"/>
+      <c r="P28" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q28" t="inlineStr"/>
+      <c r="R28" t="inlineStr"/>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>sales.enterprise@napinfo.co.id</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr"/>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Enterprise Sales</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Matrix NAP Info</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>web_research: https://napinfo.co.id/highlights/article/id/matrix-nap-info-jalin-kerja-sama-strategis-dengan-digital-realty-bersama-untuk-perkuat-ekosistem-infrastruktur-digital-nasional — Matrix NAP Info partnered with Digital Realty Bersama to strengthen Jakarta data center interconnection at its Matrix Data Center, citing rising data center, cloud, and AI computing demand as the driver.</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
+        <v>1</v>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>1a08a33c0e9b8bee</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr"/>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:23:50+00:00</t>
+        </is>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>2026-09-10T07:24:05+00:00</t>
+        </is>
+      </c>
+      <c r="N29" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O29" t="inlineStr"/>
+      <c r="P29" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q29" t="inlineStr"/>
+      <c r="R29" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Batch 7: research + send 2 more Indonesia prospects, flag 1 for review
WebFetch blocked again, Scout worked WebSearch-only across a widened net
(mining, insurance, healthcare, banking, logistics, government, telecom)
after the last two batches' yield dropped as obvious candidates ran out.
3 of ~30 companies evaluated had real, domain-matched emails; 1 of those
(Astra International) is held back in needs_manual_verification.csv —
its email domain (ai.astra.co.id) wasn't independently confirmed on a
first-party page and the underlying evidence was a stale 2023 JV
announcement, below this campaign's current-need bar. Sent the other 2
(Moratelindo, XL Axiata) live via Gmail. CRM now at 30 sent total.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R29"/>
+  <dimension ref="A1:R31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2452,6 +2452,154 @@
       <c r="Q29" t="inlineStr"/>
       <c r="R29" t="inlineStr"/>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>corpsec@xl.co.id</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Dian Siswarini</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>President Director &amp; CEO</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>XL Axiata</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>web_research: https://www.datacenterdynamics.com/en/news/princeton-digital-group-to-acquire-majority-stake-in-xl-axiatas-indonesian-data-centers/ — Princeton Digital Group agreed to acquire a 70% stake in XL Axiata data center portfolio (5 sites: Pekanbaru, Cibitung, Surabaya, Bintaro, Bandung), with PDG committing US$100M growth capital to expand capacity of the existing facilities XL Axiata co-owns</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
+        <v>1</v>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>1a08f5c3a0d23cf2</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr"/>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>2026-09-11T07:26:08+00:00</t>
+        </is>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>2026-09-11T07:26:24+00:00</t>
+        </is>
+      </c>
+      <c r="N30" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O30" t="inlineStr"/>
+      <c r="P30" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q30" t="inlineStr"/>
+      <c r="R30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>info@morarepublic.co.id</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Jimmy Kadir</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Direktur Utama &amp; CEO</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Moratelindo</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>web_research: https://www.morarepublic.co.id/our-company/news/moratelindo-dan-my-republic-indonesia-umumkan-merger-untuk-percepatan-dan-pemerataan-ekosistem-digital-di-indonesia — Merged with MyRepublic Indonesia in April 2026 to form PT Ekamas Mora Republik Tbk, combining six existing data centers (3.3MW total capacity) and national fiber networks to scale digital infrastructure and avoid capex duplication, per CEO Jimmy Kadir</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
+        <v>1</v>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>1a08f5c18cb38e73</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr"/>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>2026-09-11T07:26:08+00:00</t>
+        </is>
+      </c>
+      <c r="M31" t="inlineStr">
+        <is>
+          <t>2026-09-11T07:26:16+00:00</t>
+        </is>
+      </c>
+      <c r="N31" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="O31" t="inlineStr"/>
+      <c r="P31" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="Q31" t="inlineStr"/>
+      <c r="R31" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix XL Axiata bounce status, log batch 8 (0 verified emails, 7 form-only)
corpsec@xl.co.id bounced (550 5.1.0 address not found) despite passing
domain-match audit — the mailbox itself doesn't exist even though the
domain is real. CRM corrected from sent to bounced.

Batch 8 (on-demand, no daily schedule) evaluated ~22 more Indonesian
companies and found zero with a verifiable, domain-matched email —
several near-miss lookalike domains (dss.co.id vs dssa.co.id, bakrie.co.id
vs bakrie-brothers.com, iforte.co.id vs iforte.id) were correctly rejected
rather than guessed. 7 real leads queued contact-form-only.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -2490,28 +2490,24 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>sent</t>
+          <t>bounced</t>
         </is>
       </c>
       <c r="I30" t="n">
         <v>1</v>
       </c>
-      <c r="J30" t="inlineStr">
-        <is>
-          <t>1a08f5c3a0d23cf2</t>
-        </is>
-      </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="J30" t="inlineStr"/>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>550 5.1.0 address not found (mailer-daemon)</t>
+        </is>
+      </c>
       <c r="L30" t="inlineStr">
         <is>
           <t>2026-09-11T07:26:08+00:00</t>
         </is>
       </c>
-      <c r="M30" t="inlineStr">
-        <is>
-          <t>2026-09-11T07:26:24+00:00</t>
-        </is>
-      </c>
+      <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
           <t>none</t>

</xml_diff>

<commit_message>
Batch 9: multi-contact outreach live, 12 sent to named senior contacts
First run of the updated multi-contact approach: Scout found 5 new
companies plus 6 additional real named senior contacts at companies
already in the pipeline (BCA, BRIN, IOH, UGM, BNI, BRI), each getting a
separate, individually-addressed email instead of a CC blast. 12 of 13
new rows passed audit and were sent live (CEO/President Director/IT
Director/VP-level contacts at GoTo, Bank Mandiri, Telkom Indonesia, BCA,
BNI, BRI, IOH, plus Komdigi and BRIN). 1 flagged: Telkomsel's email domain
(telkomsel.co.id) didn't match its own listed website (telkomsel.com),
the same near-miss-domain pattern as past bad rows, held in
needs_manual_verification.csv rather than sent. CRM now at 41 sent + 1
bounced (41/42 real).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S31"/>
+  <dimension ref="A1:S43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2751,6 +2751,954 @@
       <c r="R31" t="inlineStr"/>
       <c r="S31" t="inlineStr"/>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>corporate.secretary@bankmandiri.co.id</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Timothy Utama</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Director of Information Technology</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Bank Mandiri</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>https://www.bankmandiri.co.id</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>web_research: https://investortrust.id/financial/55633/perkuat-digitalisasi-bank-mandiri-siapkan-capex-it-rp-3-triliun-di-2025 — IT Director Timothy Utama announced Rp3 trillion 2025 IT capex directed at strengthened IT infrastructure and networks, alongside the new Mandiri Digital Tower housing the bank's IT/data center operations.</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J32" t="n">
+        <v>1</v>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>1a091f9ccd394c53</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr"/>
+      <c r="M32" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N32" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:37:45+00:00</t>
+        </is>
+      </c>
+      <c r="O32" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P32" t="inlineStr"/>
+      <c r="Q32" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R32" t="inlineStr"/>
+      <c r="S32" t="inlineStr"/>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>corporate.secretary@ioh.co.id</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Vikram Sinha</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>President Director and CEO</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Indosat Ooredoo Hutchison</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>https://ioh.co.id</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>web_research: https://www.nokia.com/newsroom/indosat-ooredoo-group-nokia-and-nvidia-launch-zankore-by-indosat-ready-to-serve-the-region-with-full-stack-ai-infra-platform/ — CEO Vikram Sinha launched Zankore by Indosat, targeting 1 gigawatt of NVIDIA DGX AI Factory capacity (~200MW online 1H2027 on NVIDIA GB300 NVL72 systems) across centralized GPU infrastructure and AI data centers.</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J33" t="n">
+        <v>1</v>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>1a091fac15d07b04</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr"/>
+      <c r="M33" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N33" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:38:48+00:00</t>
+        </is>
+      </c>
+      <c r="O33" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P33" t="inlineStr"/>
+      <c r="Q33" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R33" t="inlineStr"/>
+      <c r="S33" t="inlineStr"/>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>corporate_comm@telkom.co.id</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Nanang Hendarno</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Direktur Network &amp; IT Solution (Director of Network &amp; IT Solutions)</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>Telkom Indonesia</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>https://www.telkom.co.id</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>web_research: https://www.telkom.co.id/sites/berita/id_ID/news/telkomgroup-siap-operasikan-hyperscale-data-center-neutradc-nxera-batam-dukung-ekosistem-ai-3387 — TelkomGroup preparing to operate the NeutraDC Nxera Batam hyperscale data center to support Indonesia's AI ecosystem, part of network/IT infrastructure expansion overseen by the Director of Network &amp; IT Solutions.</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J34" t="n">
+        <v>1</v>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>1a091fa278587d7c</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr"/>
+      <c r="M34" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N34" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:38:08+00:00</t>
+        </is>
+      </c>
+      <c r="O34" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P34" t="inlineStr"/>
+      <c r="Q34" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R34" t="inlineStr"/>
+      <c r="S34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>humas@komdigi.go.id</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Meutya Hafid</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Menteri Komunikasi dan Digital (Minister of Communication and Digital Affairs)</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>Komdigi</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>https://www.komdigi.go.id</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>web_research: https://katadata.co.id/digital/teknologi/6815c63429082/pusat-data-nasional-beroperasi-juni-berikut-kecanggihan-dan-fungsinya — Operates Pusat Data Nasional (PDN) Cikarang, a Tier-4 national data center with 20MW electrical capacity expandable to 80MW, using a water-cooling system, described by the ministry as Indonesia's flagship integrated government data center.</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J35" t="n">
+        <v>1</v>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>1a091f995bf79daa</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr"/>
+      <c r="M35" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N35" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:37:30+00:00</t>
+        </is>
+      </c>
+      <c r="O35" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P35" t="inlineStr"/>
+      <c r="Q35" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R35" t="inlineStr"/>
+      <c r="S35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>info@ugm.ac.id</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Prof. dr. Ova Emilia, M.Med.Ed., Sp.OG(K)., Ph.D</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Rektor (Rector)</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>Universitas Gadjah Mada</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>https://ugm.ac.id</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>web_research: https://www.overclockingid.com/kemkomdigi-indosat-nvidia-dan-ugm-resmikan-pusat-ai-berbasis-universitas-pertama-di-indonesia/ — UGM, Komdigi, Indosat, and NVIDIA launched the UGM Indosat NVIDIA AI Technology Center, Indonesia's first university-based AI center, at GIK UGM in August 2026, with Rektor Ova Emilia citing UGM's ongoing AI infrastructure commitment since 2023.</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J36" t="n">
+        <v>1</v>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>1a091fae13093edc</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr"/>
+      <c r="M36" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N36" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:38:56+00:00</t>
+        </is>
+      </c>
+      <c r="O36" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P36" t="inlineStr"/>
+      <c r="Q36" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R36" t="inlineStr"/>
+      <c r="S36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>investor@telkom.co.id</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Dian Siswarini</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>President Director (Direktur Utama)</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Telkom Indonesia</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>https://www.telkom.co.id</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>web_research: https://www.telkom.co.id/sites/berita/id_ID/news/data-center-terisi-penuh-sebelum-beroperasi-telkom-percepat-ekspansi-kapasitas-neutradc-di-batam-3797 — Telkom's NeutraDC Nxera Batam hyperscale data center sold out before going operational, prompting Telkom to accelerate capacity expansion to support Indonesia's AI ecosystem.</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J37" t="n">
+        <v>1</v>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>1a091fa094171db8</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr"/>
+      <c r="M37" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N37" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:38:00+00:00</t>
+        </is>
+      </c>
+      <c r="O37" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P37" t="inlineStr"/>
+      <c r="Q37" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R37" t="inlineStr"/>
+      <c r="S37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>investor_relations@bca.co.id</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>David Formula</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Director of Information Technology</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>Bank Central Asia</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>https://www.bca.co.id</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>web_research: https://www.liputan6.com/saham/read/5467651/data-center-bca-bakal-beroperasi-pada-2025 — BCA's new Cikarang data center began full operations in 2025 as part of a High Availability System strategy combining cloud adoption, new data center construction, and AI-based data infrastructure modernization.</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J38" t="n">
+        <v>1</v>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>1a091fa4534ae567</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N38" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:38:33+00:00</t>
+        </is>
+      </c>
+      <c r="O38" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P38" t="inlineStr"/>
+      <c r="Q38" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R38" t="inlineStr"/>
+      <c r="S38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ir@bankmandiri.co.id</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Riduan</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>President Director</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>Bank Mandiri</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>https://www.bankmandiri.co.id</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>web_research: https://investor.id/finance/373950/resmikan-mandiri-digital-tower-menteri-bumn-perkuat-data-center-untuk-digitalisasi-bumn — Bank Mandiri inaugurated the 32-floor, ~70,000 sqm Mandiri Digital Tower as its new IT/data-center hub, with the Minister of SOEs calling for the bank to further strengthen its data center capacity.</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J39" t="n">
+        <v>1</v>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>1a091f9ebe0603b0</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr"/>
+      <c r="M39" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N39" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:37:53+00:00</t>
+        </is>
+      </c>
+      <c r="O39" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P39" t="inlineStr"/>
+      <c r="Q39" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R39" t="inlineStr"/>
+      <c r="S39" t="inlineStr"/>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ir@bni.co.id</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Toto Prasetio</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Direktur Teknologi dan Operasi (Director of Technology and Operations)</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>Bank Negara Indonesia</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>https://www.bni.co.id</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>web_research: https://www.cloudcomputing.id/berita/bni-transformasi-digital-ai-cloud — Director of Technology and Operations Toto Prasetio said AI and cloud adoption are key elements of BNI's digital transformation, discussed at the BNI Investor Daily Summit 2024.</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J40" t="n">
+        <v>1</v>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>1a091fafde7aa858</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr"/>
+      <c r="M40" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N40" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:39:03+00:00</t>
+        </is>
+      </c>
+      <c r="O40" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P40" t="inlineStr"/>
+      <c r="Q40" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R40" t="inlineStr"/>
+      <c r="S40" t="inlineStr"/>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>ir@bri.co.id</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Rio Hendarwan</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Vice President, PT Bank Rakyat Indonesia (Persero) Tbk</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>Bank Rakyat Indonesia</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>https://bri.co.id</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>web_research: https://www.hutamakarya.com/en/hutama-karya-lakukan-topping-off-proyek-it-center-bri-ragunan-paket-2-siap-dukung-transformasi-digital — BRI completed topping-off of the Cloud IT Center BRI Ragunan Package 2 building (Rp517B Package 1 contract with PTPP, Package 2 with Hutama Karya), a strategic national banking IT/data center; VP Rio Hendarwan said it will accelerate service digitalization.</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J41" t="n">
+        <v>1</v>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>1a091fb1a559b904</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr"/>
+      <c r="M41" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N41" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:39:11+00:00</t>
+        </is>
+      </c>
+      <c r="O41" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P41" t="inlineStr"/>
+      <c r="Q41" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R41" t="inlineStr"/>
+      <c r="S41" t="inlineStr"/>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>ir@gotocompany.com</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Patrick Walujo</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>CEO, GoTo Group</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>GoTo Group</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>https://www.gotocompany.com</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>web_research: https://www.gotocompany.com/en/news/press/goto-group-tencent-cloud-and-alibaba-cloud-sign-agreement-to-boost-cloud-infrastructure-and-nurture-local-digital-talent-in-indonesia — CEO Patrick Walujo signed 5-year cloud infrastructure agreements with Tencent Cloud and Alibaba Cloud (incl. Tencent's 3rd Indonesia data center) to strengthen GoTo's onshore data/cloud infrastructure.</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J42" t="n">
+        <v>1</v>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>1a091f9b1d90992f</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr"/>
+      <c r="M42" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N42" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:37:38+00:00</t>
+        </is>
+      </c>
+      <c r="O42" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P42" t="inlineStr"/>
+      <c r="Q42" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R42" t="inlineStr"/>
+      <c r="S42" t="inlineStr"/>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>ppid@brin.go.id</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Arif Satria</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Kepala BRIN (Head of the National Research and Innovation Agency)</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>BRIN Mahameru HPC</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>https://www.brin.go.id</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>web_research: https://www.brin.go.id/news/121592/brin-tekankan-pentingnya-high-performance-computing-mahameru-dukung-data-riset-indonesia — BRIN operates the Mahameru HPC supercomputing cluster (92 high-density nodes, NVIDIA DGX A100 GPU facility) across its Cibinong and Serpong science-park data centers, emphasized by leadership as critical national research computing infrastructure.</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J43" t="n">
+        <v>1</v>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>1a091faa52be4315</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr"/>
+      <c r="M43" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:36:51+00:00</t>
+        </is>
+      </c>
+      <c r="N43" t="inlineStr">
+        <is>
+          <t>2026-09-11T19:38:40+00:00</t>
+        </is>
+      </c>
+      <c r="O43" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P43" t="inlineStr"/>
+      <c r="Q43" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R43" t="inlineStr"/>
+      <c r="S43" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Batch 10: 7 sent to Indonesian universities with real DGX/HPC deployments
Continuing the multi-contact, named-senior-contact approach. Scout found
a high-yield vein in universities with public NVIDIA DGX/HPC procurement
and named rectors/center heads: IT Del, Universitas Brawijaya (2 contacts
- rector + AI Center head, separate rows), Telkom University, ITS,
Universitas Gunadarma, IPB University. All 7 domain-matched and sent live.
CRM now at 48 sent + 1 bounced (49 total, XL Axiata's bounce now correctly
blocked from resend after yesterday's BLOCKING_STATUSES fix).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01CySFu7WWzhybu87DvMUJmR
</commit_message>
<xml_diff>
--- a/data/crm_database.xlsx
+++ b/data/crm_database.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S43"/>
+  <dimension ref="A1:S50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3699,6 +3699,559 @@
       <c r="R43" t="inlineStr"/>
       <c r="S43" t="inlineStr"/>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>advanced-lab@apps.ipb.ac.id</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Dr. Irdika Mansur</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Head of Advanced Research Laboratory (ARLab)</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>IPB University</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>https://www.ipb.ac.id</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>web_research: https://www.ipb.ac.id/news/index/2023/09/ipb-university-has-nvidia-dgx-a100-supercomputer-with-highest-performance-technology-in-indonesia/ — ARLab acquired an NVIDIA DGX A100 supercomputer, described by ARLab head Dr. Irdika Mansur as the highest-performance AI computing technology in Indonesia at the time, used for AI model development in agriculture/bioinformatics research</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J44" t="n">
+        <v>1</v>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>1a09479806a23b0c</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr"/>
+      <c r="M44" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:14:30+00:00</t>
+        </is>
+      </c>
+      <c r="N44" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:16:32+00:00</t>
+        </is>
+      </c>
+      <c r="O44" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P44" t="inlineStr"/>
+      <c r="Q44" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R44" t="inlineStr"/>
+      <c r="S44" t="inlineStr"/>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>humas@its.ac.id</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Prof. Ir. Bambang Pramujati</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Rektor (Rector), 2024-2029</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>ITS</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>https://www.its.ac.id</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>web_research: https://www.its.ac.id/komputer/id/launching-nvidia-dgx-a100-artificial-intelligence-supercomputer-2/ai-supercomputer-2/ — Computer Engineering Dept launched an NVIDIA DGX-A100 AI supercomputer (Feb 2025), used by ITS's Center of AI and Digital Technology (AIDT) for high-performance computing research</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J45" t="n">
+        <v>1</v>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>1a09478fb98912ea</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr"/>
+      <c r="M45" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:14:30+00:00</t>
+        </is>
+      </c>
+      <c r="N45" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:15:57+00:00</t>
+        </is>
+      </c>
+      <c r="O45" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P45" t="inlineStr"/>
+      <c r="Q45" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R45" t="inlineStr"/>
+      <c r="S45" t="inlineStr"/>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>humas@ub.ac.id</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Prof. Widodo</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Rektor (Rector), 2022-2027</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>Universitas Brawijaya</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>https://www.ub.ac.id</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>web_research: https://www.itworks.id/71583/universitas-brawijaya-resmikan-ai-center.html — Inaugurated UB's AI Center (Feb 2023), which runs an NVIDIA DGX A100 supercomputer (5 petaFLOPS) for cross-disciplinary AI research, later formally opened nationally by the Minister of Communication and Digital Affairs (Jan 2025)</t>
+        </is>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J46" t="n">
+        <v>1</v>
+      </c>
+      <c r="K46" t="inlineStr">
+        <is>
+          <t>1a094781562dc995</t>
+        </is>
+      </c>
+      <c r="L46" t="inlineStr"/>
+      <c r="M46" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:14:30+00:00</t>
+        </is>
+      </c>
+      <c r="N46" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:14:57+00:00</t>
+        </is>
+      </c>
+      <c r="O46" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P46" t="inlineStr"/>
+      <c r="Q46" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R46" t="inlineStr"/>
+      <c r="S46" t="inlineStr"/>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>info@del.ac.id</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Dr. Arnaldo Marulitua Sinaga</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Rektor (Rector)</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>IT Del</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>https://www.del.ac.id</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>web_research: https://www.del.ac.id/?p=16932 — Launched AI Center (Aug 2026) with an NVIDIA DGX H200 supercomputer (up to 156.5 petaFLOPS national AI education capacity), making IT Del Indonesia's highest AI-computing-capacity education institution, per Wakil Rektor I Dr. Johannes Sianipar</t>
+        </is>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J47" t="n">
+        <v>1</v>
+      </c>
+      <c r="K47" t="inlineStr">
+        <is>
+          <t>1a09477ddd96a9aa</t>
+        </is>
+      </c>
+      <c r="L47" t="inlineStr"/>
+      <c r="M47" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:14:30+00:00</t>
+        </is>
+      </c>
+      <c r="N47" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:14:43+00:00</t>
+        </is>
+      </c>
+      <c r="O47" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P47" t="inlineStr"/>
+      <c r="Q47" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R47" t="inlineStr"/>
+      <c r="S47" t="inlineStr"/>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>info@telkomuniversity.ac.id</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Prof. Suyanto</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Rektor (Rector), 2025-2030</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Telkom University</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>https://telkomuniversity.ac.id</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G48" t="inlineStr">
+        <is>
+          <t>web_research: https://neucentrix.hk/telkom-is-the-first-user-of-the-most-advanced-ai-supercomputer-nvidia-dgx-a100-in-indonesia/ — Operates an NVIDIA DGX A100 AI supercomputer and an Artificial Intelligence Center (AIC) as a member of the government-formed Indonesia AI Research Consortium (IARC); its former AI research center chair Prof. Suyanto is now Rector</t>
+        </is>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I48" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J48" t="n">
+        <v>1</v>
+      </c>
+      <c r="K48" t="inlineStr">
+        <is>
+          <t>1a09478c7e27301d</t>
+        </is>
+      </c>
+      <c r="L48" t="inlineStr"/>
+      <c r="M48" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:14:30+00:00</t>
+        </is>
+      </c>
+      <c r="N48" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:15:44+00:00</t>
+        </is>
+      </c>
+      <c r="O48" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P48" t="inlineStr"/>
+      <c r="Q48" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R48" t="inlineStr"/>
+      <c r="S48" t="inlineStr"/>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>mediacenter@gunadarma.ac.id</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>Prof. Dr. E.S. Margianti</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Rektor (Rector)</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>Universitas Gunadarma</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>https://www.gunadarma.ac.id</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G49" t="inlineStr">
+        <is>
+          <t>web_research: https://www.hpc-hub.gunadarma.ac.id/ — Operates NVIDIA DGX-1 and DGX A100 supercomputers via its dedicated HPC/DGX development hub for AI and data-intensive research</t>
+        </is>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I49" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J49" t="n">
+        <v>1</v>
+      </c>
+      <c r="K49" t="inlineStr">
+        <is>
+          <t>1a094792988c4c06</t>
+        </is>
+      </c>
+      <c r="L49" t="inlineStr"/>
+      <c r="M49" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:14:30+00:00</t>
+        </is>
+      </c>
+      <c r="N49" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:16:19+00:00</t>
+        </is>
+      </c>
+      <c r="O49" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P49" t="inlineStr"/>
+      <c r="Q49" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R49" t="inlineStr"/>
+      <c r="S49" t="inlineStr"/>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>wayanfm@ub.ac.id</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>Prof. Ir. Wayan Firdaus Mahmudy</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>Ketua AI Center &amp; Dean, Faculty of Computer Science (FILKOM)</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>Universitas Brawijaya</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>https://www.ub.ac.id</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>Indonesia</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>web_research: https://tugujatim.id/launching-artificial-intelligence-center-universitas-brawijaya-kolaborasikan-penelitian-antar-bidang-keilmuan/ — Appointed Head of UB's AI Center (Feb 2023), which operates an NVIDIA DGX A100 supercomputer (5 petaFLOPS) for AI/data-science research</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>legitimate_interest_b2b_public_contact</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>sent</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>1</v>
+      </c>
+      <c r="K50" t="inlineStr">
+        <is>
+          <t>1a094784229ff481</t>
+        </is>
+      </c>
+      <c r="L50" t="inlineStr"/>
+      <c r="M50" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:14:30+00:00</t>
+        </is>
+      </c>
+      <c r="N50" t="inlineStr">
+        <is>
+          <t>2026-09-12T07:15:31+00:00</t>
+        </is>
+      </c>
+      <c r="O50" t="inlineStr">
+        <is>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="P50" t="inlineStr"/>
+      <c r="Q50" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="R50" t="inlineStr"/>
+      <c r="S50" t="inlineStr"/>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>